<commit_message>
update enemies waves and dishs cooking time
</commit_message>
<xml_diff>
--- a/Assets/Configs/Dishs.xlsx
+++ b/Assets/Configs/Dishs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\Project\Project3D\Assets\Configs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Assignment\FoodGuardian\Project3D\Assets\Configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64FBA159-AF7E-4ECE-976E-2D48027DA658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CA4F8C7-3F38-42E0-ABA1-EEFBBC4E8A64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,9 +26,6 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -130,13 +127,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Yu Gothic"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Yu Gothic"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -144,7 +141,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Yu Gothic"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -454,16 +451,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="2" width="8.625" style="1"/>
+    <col min="1" max="2" width="8.59765625" style="1"/>
     <col min="3" max="3" width="9" style="1"/>
-    <col min="4" max="4" width="8.625" style="1"/>
-    <col min="5" max="5" width="44.625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="37.75" customWidth="1"/>
+    <col min="4" max="4" width="8.59765625" style="1"/>
+    <col min="5" max="5" width="44.59765625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="37.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -483,7 +480,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
         <v>6</v>
       </c>
@@ -503,7 +500,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
         <v>7</v>
       </c>
@@ -511,7 +508,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D3" s="1">
         <v>104</v>
@@ -523,7 +520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" s="1">
         <v>8</v>
       </c>
@@ -531,7 +528,7 @@
         <v>10</v>
       </c>
       <c r="C4" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D4" s="1">
         <v>105</v>
@@ -543,7 +540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
         <v>9</v>
       </c>
@@ -551,7 +548,7 @@
         <v>12</v>
       </c>
       <c r="C5" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D5" s="1">
         <v>106</v>
@@ -563,7 +560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
         <v>10</v>
       </c>
@@ -571,7 +568,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D6" s="1">
         <v>107</v>
@@ -583,7 +580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
         <v>11</v>
       </c>
@@ -603,7 +600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>12</v>
       </c>
@@ -623,7 +620,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <v>13</v>
       </c>
@@ -631,7 +628,7 @@
         <v>20</v>
       </c>
       <c r="C9" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D9" s="1">
         <v>205</v>
@@ -643,7 +640,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <v>14</v>
       </c>
@@ -651,7 +648,7 @@
         <v>23</v>
       </c>
       <c r="C10" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" s="1">
         <v>206</v>
@@ -663,7 +660,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <v>100</v>
       </c>

</xml_diff>

<commit_message>
new updates for waves and new item
</commit_message>
<xml_diff>
--- a/Assets/Configs/Dishs.xlsx
+++ b/Assets/Configs/Dishs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Unity\Project\Project3D\Assets\Configs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Assignment\FoodGuardian\Project3D\Assets\Configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0050E2-22F5-46A6-AC2D-D0F412174D4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63DD126A-13A9-42DA-A9F7-65699D73AF77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,15 +26,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>DishID</t>
   </si>
@@ -102,16 +99,10 @@
     <t>Icons/beafsoup_icon</t>
   </si>
   <si>
-    <t>13001;0.5|14001;5</t>
-  </si>
-  <si>
     <t>葱鸡腿</t>
   </si>
   <si>
     <t>Icons/Onionchicken_icon</t>
-  </si>
-  <si>
-    <t>13001;1|14001;5</t>
   </si>
   <si>
     <t>CookTime</t>
@@ -123,6 +114,22 @@
   </si>
   <si>
     <t>Icons/Junk_icon</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>满汉全席</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>13001;0.5|14001;5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>13001;1|14001;5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>13001;2|14001;5|13002;1</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -130,17 +137,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Yu Gothic"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Yu Gothic"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -148,7 +155,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Yu Gothic"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -156,10 +163,23 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Yu Gothic"/>
       <family val="2"/>
       <charset val="128"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Noto Sans JP"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="2">
@@ -182,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -191,6 +211,13 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -468,17 +495,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="2" width="8.625" style="1"/>
+    <col min="1" max="2" width="8.59765625" style="1"/>
     <col min="3" max="3" width="9" style="1"/>
-    <col min="4" max="4" width="8.625" style="1"/>
-    <col min="5" max="5" width="44.625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="37.75" customWidth="1"/>
+    <col min="4" max="4" width="8.59765625" style="1"/>
+    <col min="5" max="5" width="44.59765625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="37.69921875" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -486,7 +513,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -494,11 +521,11 @@
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
         <v>6</v>
       </c>
@@ -514,11 +541,11 @@
       <c r="E2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
         <v>7</v>
       </c>
@@ -534,11 +561,11 @@
       <c r="E3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" s="1">
         <v>8</v>
       </c>
@@ -554,11 +581,11 @@
       <c r="E4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
         <v>9</v>
       </c>
@@ -574,11 +601,11 @@
       <c r="E5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
         <v>10</v>
       </c>
@@ -594,11 +621,11 @@
       <c r="E6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" s="1">
         <v>11</v>
       </c>
@@ -614,11 +641,11 @@
       <c r="E7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>12</v>
       </c>
@@ -634,11 +661,11 @@
       <c r="E8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" s="1">
         <v>13</v>
       </c>
@@ -654,16 +681,16 @@
       <c r="E9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F9" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" s="1">
         <v>14</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C10" s="1">
         <v>4</v>
@@ -672,29 +699,46 @@
         <v>206</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A11" s="1">
+        <v>15</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="1">
+        <v>8</v>
+      </c>
+      <c r="D11" s="1">
+        <v>207</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A12" s="1">
+        <v>100</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="18.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="1">
-        <v>100</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="1">
+      <c r="C12" s="1">
         <v>3</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D12" s="1">
         <v>203</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F11" s="1">
+      <c r="E12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F12" s="6">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updates for attack speed & dish's buffs
</commit_message>
<xml_diff>
--- a/Assets/Configs/Dishs.xlsx
+++ b/Assets/Configs/Dishs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Assignment\FoodGuardian\Project3D\Assets\Configs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAA1EAB8-031D-4C56-8BB2-8BB98FA22D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F303BE4-DBB4-429B-8FF1-BDDAA06D6A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -118,19 +118,19 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>13001;2|14001;5|13003;30</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>13001;2|14001;5|13003;20</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>13001;0.5|14001;5|13003;5</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>13001;1|14001;5|13003;5</t>
+    <t>13001;2|14001;5|13004;10</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>13001;1|14001;5|13004;5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>13001;2|14001;5|13003;30|13004;30</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -683,7 +683,7 @@
         <v>20</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
@@ -703,7 +703,7 @@
         <v>22</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
@@ -720,7 +720,7 @@
         <v>207</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.45">

</xml_diff>